<commit_message>
re-export abp iteration bfs reverse
</commit_message>
<xml_diff>
--- a/experiments/results/abp/iteration-bfs-reverse/abp-sat-iteration-bfs-reverse.xlsx
+++ b/experiments/results/abp/iteration-bfs-reverse/abp-sat-iteration-bfs-reverse.xlsx
@@ -11947,7 +11947,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>45000</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -11973,28 +11973,32 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>849</t>
+          <t>870</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>905</t>
+          <t>871</t>
         </is>
       </c>
       <c r="K25" t="n">
-        <v>904</v>
+        <v>870</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>30024.3</t>
+          <t>31066.3</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>82322</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr"/>
+          <t>165074</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>